<commit_message>
feat(templates+doc): 유심 최종 정책 반영 (3사 × 3종 = 9행)
최종 유심 요금제 (매장/온라인 구조 동일 · 페이백 값만 다름):
- SK (33/45/55): 5GX 슬림 / 베이직 플러스 / 5GX 레귤러
- KT (37/50/69): 5G 슬림 / 5G 심플 / 5G 비디오
- LG (33/61/85): 5G 슬림+ / 5G 스탠다드 / 5G 프리미어 레귤러

템플릿:
- 오프라인/온라인 모두 9행 · 페이백 값은 어드민 등록 (빈칸 회색)
- 📋 안내 시트에 9종 요금제 목록 전체 기재
- flow-store-price.html 매트릭스 유심 정책 팁에도 9종 반영

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/template-offline-form.xlsx
+++ b/docs/template-offline-form.xlsx
@@ -609,7 +609,7 @@
       <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2. 컬럼은 고정 · 새 기종/요금제는 "행(Row) 추가"로 관리</t>
+          <t>2. 컬럼 고정 · 새 기종/요금제는 "행 추가"로 관리</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>3. PK = (통신사 + 모델명 + 요금제) — 업로드 시 동일 조합 덮어쓰기</t>
+          <t>3. PK = (통신사+모델명+요금제) · 업로드 시 동일 조합 덮어쓰기</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>· 무선(휴대폰): 3사 × 18종 = 54행</t>
+          <t>· 무선(휴대폰): 3사 × 18종 = 54행 (정리3 원본)</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       <c r="A11" s="2" t="inlineStr"/>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>· 유심: 3사 × 요금제별 = 8행 (SK 3 + KT 2 + LG 3) — 매장/온라인 구조 동일, 페이백 값만 다름</t>
+          <t>· 유심: 3사 × 3종 = 9행 (매장/온라인 구조 동일, 페이백 값만 다름)</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       <c r="A13" s="2" t="inlineStr"/>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>📇 통신사별 유심 요금제</t>
+          <t>📇 통신사별 유심 요금제 (3사 × 3종 = 9개)</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       <c r="A14" s="2" t="inlineStr"/>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>· SK: 세이브 / T플랜 안심2.5G / 5G 슬림</t>
+          <t>· SK: 5GX 슬림(33,000) / 베이직 플러스(45,000) / 5GX 레귤러(55,000)</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       <c r="A15" s="2" t="inlineStr"/>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>· KT: 5G 슬림 4GB / 5G 심플 30GB</t>
+          <t>· KT: 5G 슬림(37,000) / 5G 심플(50,000) / 5G 비디오(69,000)</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       <c r="A16" s="2" t="inlineStr"/>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>· LG: 데이터33 / 심플+ / 5G 에센셜</t>
+          <t>· LG: 5G 슬림+(33,000) / 5G 스탠다드(61,000) / 5G 프리미어 레귤러(85,000)</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>· 오프라인: 12개 매장 각자 복사해서 사용 · 온라인: 통합 1개</t>
+          <t>· 오프라인: 12개 매장 각자 복사 · 온라인: 통합 1개</t>
         </is>
       </c>
     </row>
@@ -2669,13 +2669,13 @@
         <v>70</v>
       </c>
     </row>
-    <row r="58" ht="75" customHeight="1">
+    <row r="58" ht="80" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>※ 번이/기변 (만원) = 공시지원금 기준 현금완납가 · 음수=페이백(초록) · 양수=부담(빨강)
-※ 인터넷/인터넷+TV (만원) = 결합 가입 시 추가 혜택 (전 행 공통 · 초록 배경)
+          <t>※ 번이/기변(만원) = 공시지원금 기준 현금완납가 · 음수=페이백(초록) · 양수=부담(빨강)
+※ 인터넷/인터넷+TV(만원) = 결합 가입 시 추가 혜택 (전 행 공통 · 초록 배경)
 ※ 요금제: SK 프리미엄 · KT 초이스스페셜 · LG 프리미어 슈퍼
-※ PK = (통신사+모델명+요금제) · 새 기종은 행 추가</t>
+※ PK=(통신사+모델명+요금제) · 새 기종은 행 추가</t>
         </is>
       </c>
     </row>
@@ -2694,13 +2694,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -2710,7 +2710,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>📇 유심 시세 — 오프라인 · 3사 × 요금제별 = 8행 (SK 3 + KT 2 + LG 3)</t>
+          <t>📇 유심 시세 — 오프라인 · 3사 × 3종 = 9행</t>
         </is>
       </c>
     </row>
@@ -2774,12 +2774,10 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>세이브 (33,000)</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="n">
-        <v>-40</v>
-      </c>
+          <t>5GX 슬림 (33,000)</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr"/>
       <c r="F3" s="14" t="inlineStr"/>
       <c r="G3" s="10" t="n">
         <v>40</v>
@@ -2806,7 +2804,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>T플랜 안심2.5G (43,890)</t>
+          <t>베이직 플러스 (45,000)</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr"/>
@@ -2836,7 +2834,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>5G 슬림 (55,000)</t>
+          <t>5GX 레귤러 (55,000)</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr"/>
@@ -2866,12 +2864,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>5G 슬림 4GB (45,000)</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>-15</v>
-      </c>
+          <t>5G 슬림 (37,000)</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="10" t="n">
         <v>40</v>
@@ -2898,7 +2894,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>5G 심플 30GB (69,000)</t>
+          <t>5G 심플 (50,000)</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr"/>
@@ -2911,9 +2907,9 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>LG</t>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>KT</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -2928,12 +2924,10 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>데이터33 (33,000)</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>-15</v>
-      </c>
+          <t>5G 비디오 (69,000)</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
       <c r="G8" s="10" t="n">
         <v>40</v>
@@ -2960,12 +2954,10 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>심플+ (43,890)</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>-30</v>
-      </c>
+          <t>5G 슬림+ (33,000)</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
       <c r="G9" s="10" t="n">
         <v>40</v>
@@ -2992,12 +2984,10 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>5G 에센셜 (55,000)</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>-40</v>
-      </c>
+          <t>5G 스탠다드 (61,000)</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
       <c r="G10" s="10" t="n">
         <v>40</v>
@@ -3006,20 +2996,51 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" ht="75" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>※ 매장·온라인 구조 동일 (8행) — 페이백 값만 다름 · 회색 셀은 어드민 등록 필요
-※ SK: 세이브 / T플랜 안심2.5G / 5G 슬림  |  KT: 5G 슬림 4GB / 5G 심플 30GB  |  LG: 데이터33 / 심플+ / 5G 에센셜
-※ MNP 전용 · 010 신규 제외 · 기변 공란 (유심은 번이만)
-※ 선택약정 25% 할인 (SK/KT 개통시 · LG 개통 후 고객센터 신청) · 실납 = 월요금 × 0.75
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>LG</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>유심-매장</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>유심-매장</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>5G 프리미어 레귤러 (85,000)</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr"/>
+      <c r="F11" s="14" t="inlineStr"/>
+      <c r="G11" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>※ 매장·온라인 구조 동일 (9행) — 페이백 값만 다름 · 빈칸(회색)=어드민 등록
+※ SK: 5GX 슬림(33,000) / 베이직 플러스(45,000) / 5GX 레귤러(55,000)
+※ KT: 5G 슬림(37,000) / 5G 심플(50,000) / 5G 비디오(69,000)
+※ LG: 5G 슬림+(33,000) / 5G 스탠다드(61,000) / 5G 프리미어 레귤러(85,000)
+※ MNP 전용 · 010 신규 제외 · 기변 공란 · 선택약정 25% 할인 (SK/KT 개통시·LG 고객센터)
 ※ 유심비: SK/LG 다음 달 청구 · KT 선납(사은품 차감) · 유지기간: SK M+6 / KT·LG 183일</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>